<commit_message>
feat: implement UI design system and establish foundational CRM component architecture
</commit_message>
<xml_diff>
--- a/汽車美容報價列表.xlsx
+++ b/汽車美容報價列表.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a34716308bfbc7e9/文件/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\car-shop-projects\car-shop-crm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{5CC11843-D75C-0246-A3D2-96A89AA54864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24C0DF06-F180-4427-B79D-609774625D1B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE3B195E-5501-4BDD-9868-6E92F686D691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{37B91F95-50B9-0445-B5F6-14F83EB95CBB}"/>
+    <workbookView xWindow="1600" yWindow="910" windowWidth="16180" windowHeight="9180" activeTab="1" xr2:uid="{37B91F95-50B9-0445-B5F6-14F83EB95CBB}"/>
   </bookViews>
   <sheets>
     <sheet name="報價單S尺寸" sheetId="7" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="套裝" sheetId="2" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191028"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -586,10 +587,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>